<commit_message>
docs(thesis): repair final package validation
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" r:id="R3f6d40d001524dfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Requirements" sheetId="2" r:id="R39fc1be70ae049b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-2_RAG-Cube" sheetId="3" r:id="Rfe3d4baf2d6b4e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-3_Factor_Position" sheetId="4" r:id="Ra88ab8f562794dc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="5" r:id="Rd5036c2fdf4549d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-2_Backbone" sheetId="6" r:id="Rc66a42414ff34f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-3_Runtime" sheetId="7" r:id="Rf258ef25c1304268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-4_Record_Fields" sheetId="8" r:id="R997c33727843443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Dataset" sheetId="9" r:id="R67d64d19aed74b77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Config_Scores" sheetId="10" r:id="Rb6199382ab204289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_HyDE" sheetId="11" r:id="R8ffa7db132184cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_CAD" sheetId="12" r:id="R22cabc606cae4d28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_SCD_Config" sheetId="13" r:id="Rb731e2d958724ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_SCD_Paired" sheetId="14" r:id="R41b64b5ab8b04f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="15" r:id="R1fc6779c52a3478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="16" r:id="Rd9ccb94aac664ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="17" r:id="Rfae8f98465334b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" r:id="R10480c9522014738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Requirements" sheetId="2" r:id="R692cd9b1afdb4d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-2_RAG-Cube" sheetId="3" r:id="Rfb5b705026d846c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-3_Factor_Position" sheetId="4" r:id="Re19b5740631b4b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="5" r:id="R4cdac8a60274422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-2_Backbone" sheetId="6" r:id="R8957e3a709c54e1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-3_Runtime" sheetId="7" r:id="R06aee1cffe434be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-4_Record_Fields" sheetId="8" r:id="Re64e4fe2f54c43a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Dataset" sheetId="9" r:id="Rc02fe8ffda294e29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Config_Scores" sheetId="10" r:id="R67a64b4fd8a84195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_HyDE" sheetId="11" r:id="R8274cbfe982641cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_CAD" sheetId="12" r:id="R9a68d33155284b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_SCD_Config" sheetId="13" r:id="R6a7a7ac77771465f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_SCD_Paired" sheetId="14" r:id="R384fe1841817417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="15" r:id="R807ec1ae130e4443"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="16" r:id="R6ad21f93871741ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="17" r:id="Radd17ac0367d4d48"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -646,7 +646,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/GRADUATION_REPORT_TRANSFER_KO_60Q.md</x:v>
+        <x:v>출처: FINALDOCS/MANUSCRIPT/GRADUATION_REPORT_TRANSFER_KO_60Q.md</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" hidden="0" customHeight="1">
@@ -754,7 +754,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1998a2819a444fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaa1c3ed0c004329"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -779,7 +779,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/rag_cube_config_scores_60q.csv</x:v>
+        <x:v>출처: experiments/results/analysis/extended_validation_60_analysis.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" hidden="0" customHeight="1">
@@ -996,7 +996,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bee99218bff4f2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd836b576de4f4f77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1021,7 +1021,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/hyde_primary_60q.csv</x:v>
+        <x:v>출처: experiments/results/analysis/extended_validation_60_analysis.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" hidden="0" customHeight="1">
@@ -1146,7 +1146,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79046a6b4e6b4ec1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c1ca1aa083a46c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1171,7 +1171,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/cad_primary_60q.csv</x:v>
+        <x:v>출처: experiments/results/analysis/extended_validation_60_analysis.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" hidden="0" customHeight="1">
@@ -1296,7 +1296,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5e65fa6ec04b25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfec9e1c830144cb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1323,7 +1323,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/scd_language_summary_60q.csv</x:v>
+        <x:v>출처: experiments/results/analysis/extended_validation_60_analysis.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1478,7 +1478,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a92c8922d204fad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bb213b3fd1d4056"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1562,7 +1562,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9fec9068ae2493b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf544963e20d9447d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2816,7 +2816,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5553328a9334f0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1555dab508214d03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2839,7 +2839,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/paper_level_exploratory_60q.csv</x:v>
+        <x:v>출처: experiments/results/analysis/extended_validation_60_analysis.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -3410,7 +3410,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Readb90149f304f4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72b5e33ede414520"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3433,7 +3433,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/query_type_exploratory_60q.csv</x:v>
+        <x:v>출처: experiments/results/analysis/extended_validation_60_analysis.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -4412,7 +4412,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cc60745baf842ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56c01de367b545d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4509,7 +4509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de84255ea9b4d73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc360985059eb4753"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4695,7 +4695,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R754d782388334fcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf29f06a60b0427e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4783,7 +4783,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcf3799af5d48fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c795ba38dd44171"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4885,7 +4885,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra930935caab744ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce3b2e0409ce477f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4979,7 +4979,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d62a6c865dc4b73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aa1c792e3e4489c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5001,7 +5001,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>출처: docs/PAPER/FINAL/generated/runtime_summary_60q.csv</x:v>
+        <x:v>출처: experiments/results/main_generation + experiments/results/extended_validation generation records</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -5137,7 +5137,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb54ee7022b47ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cd56157017a4dfd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5215,7 +5215,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dab4c17f87b41ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8858fa9659e0478b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5293,7 +5293,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f7c3b25a354437b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf97ebaf607140db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(thesis): synchronize revised taxonomy workbook
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -739,7 +739,6 @@
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -950,7 +949,6 @@
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -1244,7 +1242,6 @@
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -1446,7 +1443,6 @@
       <c r="F2" s="1" t="n"/>
       <c r="G2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -1654,7 +1650,6 @@
       <c r="H2" s="1" t="n"/>
       <c r="I2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -1884,7 +1879,6 @@
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -3382,7 +3376,7 @@
       </c>
       <c r="D49" s="25" t="inlineStr">
         <is>
-          <t>crosslingual_ko</t>
+          <t>simple_qa</t>
         </is>
       </c>
       <c r="E49" s="25" t="n">
@@ -3412,7 +3406,7 @@
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>decoder_ablation</t>
+          <t>section_method</t>
         </is>
       </c>
       <c r="E50" s="25" t="n">
@@ -3472,7 +3466,7 @@
       </c>
       <c r="D52" s="25" t="inlineStr">
         <is>
-          <t>numeric_or_factual_hallucination</t>
+          <t>section_result</t>
         </is>
       </c>
       <c r="E52" s="25" t="n">
@@ -3502,7 +3496,7 @@
       </c>
       <c r="D53" s="25" t="inlineStr">
         <is>
-          <t>crosslingual_ko</t>
+          <t>section_result</t>
         </is>
       </c>
       <c r="E53" s="25" t="n">
@@ -3532,7 +3526,7 @@
       </c>
       <c r="D54" s="25" t="inlineStr">
         <is>
-          <t>decoder_ablation</t>
+          <t>section_result</t>
         </is>
       </c>
       <c r="E54" s="25" t="n">
@@ -3652,7 +3646,7 @@
       </c>
       <c r="D58" s="25" t="inlineStr">
         <is>
-          <t>decoder_ablation</t>
+          <t>section_result</t>
         </is>
       </c>
       <c r="E58" s="25" t="n">
@@ -3802,7 +3796,7 @@
       </c>
       <c r="D63" s="25" t="inlineStr">
         <is>
-          <t>numeric_or_factual_hallucination</t>
+          <t>simple_qa</t>
         </is>
       </c>
       <c r="E63" s="25" t="n">
@@ -3832,7 +3826,7 @@
       </c>
       <c r="D64" s="25" t="inlineStr">
         <is>
-          <t>decoder_ablation</t>
+          <t>section_method</t>
         </is>
       </c>
       <c r="E64" s="25" t="n">
@@ -3894,7 +3888,6 @@
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -4676,7 +4669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4737,1293 +4730,765 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>HyDE</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>faithfulness</t>
         </is>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0118</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.0036</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.0016</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.125</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-0.008500000000000001</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.0478</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-0.0191</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>simple_qa</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>22</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.1097</v>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>22</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.2438</v>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>22</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.0727</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>22</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.09089999999999999</v>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>21</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.108</v>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>22</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1108</v>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>22</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>section_method</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>22</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-0.0025</v>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>20</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.0193</v>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.0016</v>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>20</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-0.0014</v>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>20</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-0.0606</v>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-0.0124</v>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>section_result</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HyDE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="38" t="n">
-        <v>0.1282</v>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="E29" t="n">
+        <v>0.0313</v>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>HyDE</t>
         </is>
       </c>
-      <c r="C6" s="25" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>answer_relevancy</t>
         </is>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D30" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="38" t="n">
-        <v>0.08989999999999999</v>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="E30" t="n">
+        <v>-0.0447</v>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>HyDE</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>context_precision</t>
         </is>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D31" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="38" t="n">
-        <v>0.0528</v>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
+      <c r="E31" t="n">
+        <v>-0.2334</v>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>HyDE</t>
         </is>
       </c>
-      <c r="C8" s="25" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>context_recall</t>
         </is>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D32" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E32" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>CAD</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>faithfulness</t>
         </is>
       </c>
-      <c r="D9" s="25" t="n">
+      <c r="D33" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="38" t="n">
-        <v>-0.0333</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="E33" t="n">
+        <v>-0.2188</v>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>CAD</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>answer_relevancy</t>
         </is>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D34" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="38" t="n">
-        <v>-0.0794</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="E34" t="n">
+        <v>-0.4501</v>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>CAD</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>context_precision</t>
         </is>
       </c>
-      <c r="D11" s="25" t="n">
+      <c r="D35" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="38" t="n">
-        <v>-0.077</v>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="25" t="inlineStr">
-        <is>
-          <t>crosslingual_ko</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>section_abstract</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>CAD</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>context_recall</t>
         </is>
       </c>
-      <c r="D12" s="25" t="n">
+      <c r="D36" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="38" t="n">
+      <c r="E36" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C13" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D13" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="38" t="n">
-        <v>-0.1266</v>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C14" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" s="38" t="n">
-        <v>0.0059</v>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C15" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" s="38" t="n">
-        <v>-0.0834</v>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C16" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C17" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D17" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" s="38" t="n">
-        <v>-0.0767</v>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B18" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C18" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D18" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="38" t="n">
-        <v>0.039</v>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C19" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D19" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>decoder_ablation</t>
-        </is>
-      </c>
-      <c r="B20" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C20" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D20" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B21" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C21" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D21" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="38" t="n">
-        <v>-0.1357</v>
-      </c>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B22" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C22" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D22" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="38" t="n">
-        <v>0.0711</v>
-      </c>
-    </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B23" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C23" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D23" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="38" t="n">
-        <v>0.0563</v>
-      </c>
-    </row>
-    <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B24" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C24" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D24" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C25" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D25" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="38" t="n">
-        <v>-0.05</v>
-      </c>
-    </row>
-    <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B26" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C26" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D26" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="38" t="n">
-        <v>-0.0606</v>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B27" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C27" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D27" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="25" t="inlineStr">
-        <is>
-          <t>numeric_or_factual_hallucination</t>
-        </is>
-      </c>
-      <c r="B28" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C28" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D28" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B29" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C29" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D29" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="38" t="n">
-        <v>0.0312</v>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B30" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D30" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="38" t="n">
-        <v>-0.0447</v>
-      </c>
-    </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B31" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C31" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D31" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="38" t="n">
-        <v>-0.2334</v>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C32" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D32" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B33" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D33" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" s="38" t="n">
-        <v>-0.2188</v>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B34" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C34" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D34" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="38" t="n">
-        <v>-0.4501</v>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C35" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D35" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E35" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="25" t="inlineStr">
-        <is>
-          <t>section_abstract</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C36" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D36" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B37" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C37" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D37" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E37" s="38" t="n">
-        <v>0.1295</v>
-      </c>
-    </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B38" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C38" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D38" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E38" s="38" t="n">
-        <v>0.2685</v>
-      </c>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C39" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D39" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E39" s="38" t="n">
-        <v>-0.0594</v>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B40" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C40" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D40" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E40" s="38" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="41" ht="24" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C41" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D41" s="25" t="n">
-        <v>19</v>
-      </c>
-      <c r="E41" s="38" t="n">
-        <v>0.1284</v>
-      </c>
-    </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C42" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D42" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E42" s="38" t="n">
-        <v>0.1157</v>
-      </c>
-    </row>
-    <row r="43" ht="24" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C43" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D43" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E43" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" ht="24" customHeight="1">
-      <c r="A44" s="25" t="inlineStr">
-        <is>
-          <t>section_method</t>
-        </is>
-      </c>
-      <c r="B44" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C44" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D44" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E44" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C45" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D45" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E45" s="38" t="n">
-        <v>0.0244</v>
-      </c>
-    </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C46" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D46" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E46" s="38" t="n">
-        <v>-0.0364</v>
-      </c>
-    </row>
-    <row r="47" ht="24" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C47" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D47" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E47" s="38" t="n">
-        <v>-0.0029</v>
-      </c>
-    </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C48" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D48" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E48" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B49" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C49" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D49" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E49" s="38" t="n">
-        <v>0.0014</v>
-      </c>
-    </row>
-    <row r="50" ht="24" customHeight="1">
-      <c r="A50" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B50" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C50" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D50" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E50" s="38" t="n">
-        <v>-0.0727</v>
-      </c>
-    </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B51" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C51" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E51" s="38" t="n">
-        <v>0.0045</v>
-      </c>
-    </row>
-    <row r="52" ht="24" customHeight="1">
-      <c r="A52" s="25" t="inlineStr">
-        <is>
-          <t>section_result</t>
-        </is>
-      </c>
-      <c r="B52" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C52" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D52" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E52" s="38" t="n">
-        <v>-0.0625</v>
-      </c>
-    </row>
-    <row r="53" ht="15" customHeight="1">
-      <c r="A53" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B53" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C53" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D53" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E53" s="38" t="n">
-        <v>0.0066</v>
-      </c>
-    </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B54" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C54" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E54" s="38" t="n">
-        <v>-0.0154</v>
-      </c>
-    </row>
-    <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C55" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E55" s="38" t="n">
-        <v>-0.0174</v>
-      </c>
-    </row>
-    <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="inlineStr">
-        <is>
-          <t>HyDE</t>
-        </is>
-      </c>
-      <c r="C56" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E56" s="38" t="n">
-        <v>-0.1429</v>
-      </c>
-    </row>
-    <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B57" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C57" s="25" t="inlineStr">
-        <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="D57" s="25" t="n">
-        <v>13</v>
-      </c>
-      <c r="E57" s="38" t="n">
-        <v>0.0094</v>
-      </c>
-    </row>
-    <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B58" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C58" s="25" t="inlineStr">
-        <is>
-          <t>answer_relevancy</t>
-        </is>
-      </c>
-      <c r="D58" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E58" s="38" t="n">
-        <v>-0.0405</v>
-      </c>
-    </row>
-    <row r="59" ht="24" customHeight="1">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B59" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C59" s="25" t="inlineStr">
-        <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E59" s="38" t="n">
-        <v>-0.0337</v>
-      </c>
-    </row>
-    <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="25" t="inlineStr">
-        <is>
-          <t>simple_qa</t>
-        </is>
-      </c>
-      <c r="B60" s="25" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="C60" s="25" t="inlineStr">
-        <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="D60" s="25" t="n">
-        <v>14</v>
-      </c>
-      <c r="E60" s="38" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="37" ht="24" customHeight="1"/>
+    <row r="38" ht="24" customHeight="1"/>
+    <row r="39" ht="24" customHeight="1"/>
+    <row r="40" ht="24" customHeight="1"/>
+    <row r="41" ht="24" customHeight="1"/>
+    <row r="42" ht="24" customHeight="1"/>
+    <row r="43" ht="24" customHeight="1"/>
+    <row r="44" ht="24" customHeight="1"/>
+    <row r="45" ht="24" customHeight="1"/>
+    <row r="46" ht="24" customHeight="1"/>
+    <row r="47" ht="24" customHeight="1"/>
+    <row r="48" ht="24" customHeight="1"/>
+    <row r="49" ht="24" customHeight="1"/>
+    <row r="50" ht="24" customHeight="1"/>
+    <row r="51" ht="24" customHeight="1"/>
+    <row r="52" ht="24" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="24" customHeight="1"/>
+    <row r="55" ht="24" customHeight="1"/>
+    <row r="56" ht="24" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="24" customHeight="1"/>
+    <row r="59" ht="24" customHeight="1"/>
+    <row r="60" ht="24" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
@@ -6068,7 +5533,6 @@
       <c r="B2" s="1" t="n"/>
       <c r="C2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -6221,7 +5685,6 @@
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -6537,7 +6000,7 @@
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>RAGAS 4개 품질 지표</t>
+          <t>RAGAS 품질 지표</t>
         </is>
       </c>
     </row>
@@ -6554,12 +6017,12 @@
       </c>
       <c r="C6" s="25" t="inlineStr">
         <is>
-          <t>동일 문맥 60 대응쌍; faithfulness 58 완결쌍</t>
+          <t>동일 문맥 60 대응쌍; faithfulness 58 유효쌍</t>
         </is>
       </c>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>RAGAS 4개 품질 지표</t>
+          <t>faithfulness·answer relevancy·generation duration</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6671,7 +6134,7 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>BGE-M3 dense + BM25 sparse + weighted RRF + CrossEncoder rerank</t>
+          <t>BGE-M3 dense + BM25 sparse + weighted RRF(k=60; 0.6/0.4) + cross-encoder/ms-marco-MiniLM-L-6-v2</t>
         </is>
       </c>
     </row>
@@ -6688,48 +6151,72 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>최종 문맥 수</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>chunking</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>512 tokens / overlap 64 / minimum 50</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>max_new_tokens</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="inlineStr">
-        <is>
-          <t>512</t>
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>문맥 길이 관리</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>ContextCompressor extractive; max 3072 tokens; ratio 0.5</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>CAD alpha</t>
+          <t>최종 문맥 수</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
+          <t>max_new_tokens</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>512</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>CAD alpha</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
           <t>SCD</t>
         </is>
       </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>reference_scd; alpha=1.1, beta=0.9, Tstart=5</t>
         </is>
@@ -6833,7 +6320,7 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>CrossEncoder reranking</t>
+          <t>cross-encoder/ms-marco-MiniLM-L-6-v2</t>
         </is>
       </c>
     </row>
@@ -6845,7 +6332,7 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>rerank 결과에서 상위 5개 context</t>
+          <t>ContextCompressor 문맥 길이 관리 후 rerank 상위 5개 context</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6407,6 @@
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -7112,7 +6598,6 @@
       </c>
       <c r="B2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -7226,7 +6711,6 @@
       </c>
       <c r="B2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Apply confirmed thesis prose revisions and verify Hancom outputs
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="T2-1_Related_Work" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T3-1_Requirements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="T3-2_RAG-Cube" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="T3-3_Factor_Position" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="T4-1_Environment" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="T4-2_Backbone" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="T4-3_Runtime" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="T4-4_Record_Fields" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="T5-1_Dataset" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="T5-2_Config_Scores" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="T5-3_HyDE" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="T5-4_CAD" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="T5-5_SCD_Config" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="T5-6_SCD_Paired" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Appendix_Queries" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Appendix_Paper" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Appendix_QueryType" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Requirements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-2_RAG-Cube" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-3_Factor_Position" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-2_Backbone" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-3_Runtime" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-4_Record_Fields" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Dataset" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Config_Scores" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_HyDE" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_CAD" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_SCD_Config" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_SCD_Paired" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +80,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -102,11 +102,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -123,6 +129,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -538,22 +550,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>밀집 검색</t>
+          <t>밀집 검색과 검색 평가</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>DPR[10], BEIR[20]</t>
+          <t>DPR[11], BEIR[20]</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>한국어 질의와 영어 문장 사이의 검색 표현 간극을 HyDE 조건으로 관찰</t>
+          <t>한국어 질의와 영어 문서 사이의 검색 표현 차이를 HyDE 조건으로 비교</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>본 연구의 고정 백본 적용 범위</t>
+          <t>DPR은 검색 방법, BEIR은 관련 평가 연구로 참조</t>
         </is>
       </c>
     </row>
@@ -565,17 +577,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>FiD[11], 긴 문맥 분석[12]</t>
+          <t>FiD[12], 긴 문맥 분석[9]</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>rerank된 상위 5개 문맥을 고정해 answer/context 지표를 분리</t>
+          <t>재정렬 순위에 따라 상위 5개 청크를 선택하고 답변 지표와 문맥 지표를 구분</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>문맥 길이와 순서 정책은 고정</t>
+          <t>문맥 수와 순서 정책 고정</t>
         </is>
       </c>
     </row>
@@ -614,19 +626,19 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>같은 입력에서 C1/C0 대응 비교</t>
+          <t>같은 질의와 검색 문맥에서 C1/C0 주 비교</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>CAD α=0.5 고정 조건</t>
+          <t>CAD ON 조건의 alpha=0.5 고정</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>교정·자기검증 RAG</t>
+          <t>교정 및 자기검증 RAG</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -636,7 +648,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>검색·생성·출력 문제를 별도 층위로 해석하는 관점</t>
+          <t>검색, 생성과 출력 언어의 문제를 구분하여 설명</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -653,12 +665,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>RAGAS[9], RAG survey[19]</t>
+          <t>RAGAS[10], RAG survey[19]</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>근거 충실도·답변 관련성·문맥 정밀도·문맥 재현율 평가</t>
+          <t>근거 충실도, 답변 관련성, 문맥 정밀도와 문맥 재현율 평가</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -709,7 +721,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>[SCD OFF — 영어 검색 문맥 평가]</t>
         </is>
@@ -859,7 +871,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>[SCD ON — 한국어 변환 평가 문맥]</t>
         </is>
@@ -1009,7 +1021,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>[표 5-2 주석] 두 평가 프로토콜 블록은 각 평가 문맥 구성 방식 안에서 조건별 기술통계로 해석한다. SCD의 주 비교는 표 5-5와 표 5-6의 한국어 문자 비율 대응 결과를 사용한다.</t>
         </is>
@@ -1073,7 +1085,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>평균 변화 ON−OFF</t>
+          <t>평균 대응 차이 ON−OFF</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1263,7 +1275,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>평균 변화 ON−OFF</t>
+          <t>평균 대응 차이 ON−OFF</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1349,7 +1361,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>[진단값] 동일 검색 입력에서 자동 평가 모델 값 차이: 문맥 정밀도 8/60쌍, 문맥 재현율 1/60쌍</t>
         </is>
@@ -1423,7 +1435,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>평균 변화</t>
+          <t>평균 대응 차이</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1660,7 +1672,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>한국어 문자 비율 평균 변화</t>
+          <t>한국어 문자 비율 평균 대응 차이</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1814,7 +1826,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
@@ -1844,7 +1856,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
@@ -1874,7 +1886,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
@@ -1904,7 +1916,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
@@ -1934,7 +1946,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
@@ -1964,7 +1976,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
@@ -1994,7 +2006,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
@@ -2024,7 +2036,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
@@ -2054,7 +2066,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
@@ -2084,7 +2096,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
@@ -2114,7 +2126,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
@@ -2144,7 +2156,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
@@ -2174,7 +2186,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
@@ -2204,7 +2216,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -2234,7 +2246,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
@@ -2264,7 +2276,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
@@ -2294,7 +2306,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
@@ -2324,7 +2336,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
@@ -2354,7 +2366,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
@@ -2384,7 +2396,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
@@ -2414,7 +2426,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
@@ -2444,7 +2456,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
@@ -2474,7 +2486,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
@@ -2504,7 +2516,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
@@ -2534,7 +2546,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
@@ -2564,7 +2576,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
@@ -2594,7 +2606,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
@@ -2624,7 +2636,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
@@ -2654,7 +2666,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
@@ -2684,7 +2696,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -2714,7 +2726,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
@@ -2744,7 +2756,7 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
@@ -2774,7 +2786,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
@@ -2804,7 +2816,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -2834,7 +2846,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
@@ -2864,7 +2876,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
@@ -2894,7 +2906,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
@@ -2924,7 +2936,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
@@ -2954,7 +2966,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
@@ -2984,7 +2996,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
@@ -3014,7 +3026,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
@@ -3044,7 +3056,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
@@ -3074,7 +3086,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
@@ -3104,7 +3116,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
@@ -3134,7 +3146,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
@@ -3164,7 +3176,7 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
@@ -3194,7 +3206,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
@@ -3224,7 +3236,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
@@ -3254,7 +3266,7 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
@@ -3284,7 +3296,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
@@ -3314,7 +3326,7 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
@@ -3344,7 +3356,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E55" s="4" t="n">
@@ -3374,7 +3386,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E56" s="4" t="n">
@@ -3404,7 +3416,7 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
@@ -3434,7 +3446,7 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
@@ -3464,7 +3476,7 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
@@ -3494,7 +3506,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
@@ -3524,7 +3536,7 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
@@ -3554,7 +3566,7 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
@@ -3584,7 +3596,7 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
@@ -3653,12 +3665,12 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>유효쌍 수 n</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>평균 변화</t>
+          <t>평균 대응 차이</t>
         </is>
       </c>
     </row>
@@ -4455,19 +4467,19 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>유효쌍 수 n</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>평균 변화</t>
+          <t>평균 대응 차이</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -4490,7 +4502,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -4513,7 +4525,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -4536,7 +4548,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -4559,7 +4571,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -4582,7 +4594,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -4605,7 +4617,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -4628,7 +4640,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>사실·정의</t>
+          <t>사실 및 정의</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -4651,7 +4663,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -4674,7 +4686,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -4697,7 +4709,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -4720,7 +4732,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -4743,7 +4755,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -4766,7 +4778,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -4789,7 +4801,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -4812,7 +4824,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>방법·절차</t>
+          <t>방법 및 절차</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -4835,7 +4847,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -4858,7 +4870,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -4881,7 +4893,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -4904,7 +4916,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -4927,7 +4939,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -4950,7 +4962,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -4973,7 +4985,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -4996,7 +5008,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>결과·비교</t>
+          <t>결과 및 비교</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -5019,7 +5031,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -5042,7 +5054,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -5065,7 +5077,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -5088,7 +5100,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -5111,7 +5123,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -5134,7 +5146,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -5157,7 +5169,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -5180,7 +5192,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>목적·기여</t>
+          <t>목적 및 기여</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -5279,7 +5291,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>HyDE·CAD·SCD ON/OFF</t>
+          <t>HyDE, CAD, SCD의 ON/OFF</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -5678,7 +5690,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>CAD OFF·SCD OFF의 60 대응쌍</t>
+          <t>CAD와 SCD가 모두 OFF인 60개 대응쌍</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -5705,7 +5717,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>근거 충실도·답변 관련성·생성 시간</t>
+          <t>근거 충실도, 답변 관련성과 조건 실행 시간</t>
         </is>
       </c>
     </row>
@@ -5722,7 +5734,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>HyDE OFF 동일 문맥 120쌍; 전체 240 상태 일치 대응쌍</t>
+          <t>HyDE OFF 동일 문맥 120쌍; 동일 질의의 HyDE와 CAD 상태를 맞춘 전체 240쌍</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -5799,7 +5811,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>각 단계에서 확률이 가장 높은 토큰 선택</t>
+          <t>각 단계에서 최종 로짓이 가장 높은 토큰 선택</t>
         </is>
       </c>
     </row>
@@ -5830,12 +5842,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>청크 분할</t>
+          <t>일반 텍스트 청크 분할</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>공백 분리 기준 최대 512개 단어 / 64개 단어 중첩 / 최소 50개 단어</t>
+          <t>공백 분리 기준 최대 크기 512개 단어 / 중첩 크기 64개 단어 / 최소 크기 50개 단어</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5859,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ContextCompressor 추출식; 공백 분리 기준 최대 3,072개 단어; 압축 비율 0.5</t>
+          <t>ContextCompressor; 공백 분리 기준 3,072개 단어 초과 시 추출식 압축, 압축 비율 설정 0.5</t>
         </is>
       </c>
     </row>
@@ -5874,7 +5886,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CAD α</t>
+          <t>CAD ON의 α</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -5997,7 +6009,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ContextCompressor 문맥 길이 관리 후 재정렬 상위 5개 문맥</t>
+          <t>재정렬 상위 5개 청크 선택 → ContextCompressor의 조건부 추출식 압축 → 3,072개 단어 상한에 맞춘 문맥 절단</t>
         </is>
       </c>
     </row>
@@ -6021,12 +6033,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>HyDE 검색 표현 확장 / CAD·SCD 생성 제어</t>
+          <t>HyDE는 밀집 검색 입력에 적용 / CAD와 SCD는 답변 디코딩에 적용</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>[표 4-2 주석] 검색 후보 수 8, 재정렬 후보 수 8, 최종 문맥 수 5는 최종 평가 집합과 분리된 5개 튜닝 질의의 검색 폭 비교를 통해 사전에 선정한 값이다. CAD와 SCD의 파라미터는 각 기법의 실험 설정에 따라 별도로 적용하였다.</t>
         </is>
@@ -6061,7 +6073,7 @@
     <row r="1" ht="23" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>표 4-3 조건별 생성 시간</t>
+          <t>실험 조건별 실행 시간</t>
         </is>
       </c>
     </row>
@@ -6085,12 +6097,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>평균 생성 시간(초)</t>
+          <t>평균 조건 실행 시간(초)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>생성 시간 중앙값(초)</t>
+          <t>조건 실행 시간 중앙값(초)</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6314,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>retrieved_chunk_ids, reranked_chunk_ids, contexts</t>
+          <t>retrieved_chunk_ids(검색 후보 ID), reranked_chunk_ids(재정렬 후 최종 선택 청크 ID), contexts(최종 검색 문맥)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply professor acceptance audit to thesis and A1 poster
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" r:id="Rb8f37f0fe13f43ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Factorial_Design" sheetId="2" r:id="Rc4edbeb5c8ac4e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="3" r:id="R2d1691860ec74067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Mean_SD" sheetId="4" r:id="R88bf25d8ed9e4adb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Runtime_SD" sheetId="5" r:id="Rad26113e60334b03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_Quality_S0" sheetId="6" r:id="Rcc7805bbdd1d4249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_Quality_S1" sheetId="7" r:id="R7dcc3b35fe5b40d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_Factorial" sheetId="8" r:id="R44e4d028665b4782"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_Factorial" sheetId="9" r:id="R0b4a7a70c2c34e96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-7_Paired_Quality" sheetId="10" r:id="R8e369feb7ee64384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-8_Paired_Language" sheetId="11" r:id="R8b94d7c4c67e4ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="12" r:id="R9a1e64cb25954a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="13" r:id="Rf2051d52a1f14d2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="14" r:id="R1f1507d023dc40b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" r:id="R44db39e2cad547ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Factorial_Design" sheetId="2" r:id="R181d246532ba402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="3" r:id="Reaae07f6769f4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Mean_SD" sheetId="4" r:id="R28cfd973e48b477f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Runtime_SD" sheetId="5" r:id="Ra8b2ed1e3b1d4ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_Quality_S0" sheetId="6" r:id="R589fdbbea77744df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_Quality_S1" sheetId="7" r:id="Redd57846acee496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_Factorial" sheetId="8" r:id="R6e277814193d4085"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_Factorial" sheetId="9" r:id="Red3aba4d826b4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-7_Paired_Quality" sheetId="10" r:id="R00c0d7aff4034723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-8_Paired_Language" sheetId="11" r:id="R79fc39bfe19b4fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="12" r:id="R7928e6df557f4bdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="13" r:id="R44d57f462e7447b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="14" r:id="Raa0122dce4e84a9a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41,7 +41,7 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -53,8 +53,13 @@
         <x:fgColor rgb="FFE8E2F4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8E2F4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border>
       <x:left/>
       <x:right/>
@@ -77,11 +82,26 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FF695184"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -106,6 +126,15 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -326,13 +355,13 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>연구</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>핵심 접근</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>본 연구의 비교 질문</x:v>
       </x:c>
     </x:row>
@@ -431,25 +460,25 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>요인·지표</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>n</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>평균 차이(SD)</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>t(df)</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>p</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>보정 p</x:v>
       </x:c>
-      <x:c r="G3" s="6" t="str">
+      <x:c r="G3" s="10" t="str">
         <x:v>dz</x:v>
       </x:c>
     </x:row>
@@ -666,25 +695,25 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>요인·지표</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>n</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>평균 차이(SD)</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>t(df)</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>p</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>보정 p</x:v>
       </x:c>
-      <x:c r="G3" s="6" t="str">
+      <x:c r="G3" s="10" t="str">
         <x:v>dz</x:v>
       </x:c>
     </x:row>
@@ -762,22 +791,22 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="95" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>query ID</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>한국어 질문</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>대상 문서</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>유형</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>원문 페이지</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>정답 근거 구간</x:v>
       </x:c>
     </x:row>
@@ -2008,19 +2037,19 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>집단</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>요인</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>지표</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>유효 n</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>평균 차이(SD)</x:v>
       </x:c>
     </x:row>
@@ -2595,19 +2624,19 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>집단</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>요인</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>지표</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>유효 n</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>평균 차이(SD)</x:v>
       </x:c>
     </x:row>
@@ -3181,16 +3210,16 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>조건</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>S</x:v>
       </x:c>
     </x:row>
@@ -3331,13 +3360,13 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>구성 단계</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>사용 모델 또는 방법</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>주요 설정</x:v>
       </x:c>
     </x:row>
@@ -3479,22 +3508,22 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>조건</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>충실도</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>관련성</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>정밀도</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>재현율</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>한국어 비율</x:v>
       </x:c>
     </x:row>
@@ -3520,122 +3549,122 @@
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="8" t="str">
-        <x:v>H0C0S1</x:v>
+        <x:v>H0C1S0</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>0.787 (0.254)</x:v>
+        <x:v>0.839 (0.201)</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>0.637 (0.296)</x:v>
+        <x:v>0.675 (0.261)</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>0.763 (0.300)</x:v>
+        <x:v>0.740 (0.302)</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>0.900 (0.303)</x:v>
+        <x:v>0.917 (0.279)</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>0.699 (0.329)</x:v>
+        <x:v>0.488 (0.245)</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>H0C1S0</x:v>
+        <x:v>H1C0S0</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>0.839 (0.201)</x:v>
+        <x:v>0.834 (0.186)</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>0.675 (0.261)</x:v>
+        <x:v>0.763 (0.209)</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>0.740 (0.302)</x:v>
+        <x:v>0.714 (0.296)</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>0.917 (0.279)</x:v>
+        <x:v>0.933 (0.252)</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
-        <x:v>0.488 (0.245)</x:v>
+        <x:v>0.556 (0.213)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="8" t="str">
-        <x:v>H0C1S1</x:v>
+        <x:v>H1C1S0</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>0.777 (0.270)</x:v>
+        <x:v>0.860 (0.181)</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>0.600 (0.321)</x:v>
+        <x:v>0.705 (0.248)</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>0.752 (0.301)</x:v>
+        <x:v>0.736 (0.271)</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>0.850 (0.360)</x:v>
+        <x:v>0.900 (0.303)</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
-        <x:v>0.719 (0.218)</x:v>
+        <x:v>0.503 (0.229)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="8" t="str">
-        <x:v>H1C0S0</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>0.834 (0.186)</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>0.763 (0.209)</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="str">
-        <x:v>0.714 (0.296)</x:v>
-      </x:c>
-      <x:c r="E8" s="9" t="str">
-        <x:v>0.933 (0.252)</x:v>
-      </x:c>
-      <x:c r="F8" s="9" t="str">
-        <x:v>0.556 (0.213)</x:v>
+      <x:c r="A8" s="11" t="str">
+        <x:v>H0C0S1</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>0.787 (0.254)</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>0.637 (0.296)</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>0.763 (0.300)</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="str">
+        <x:v>0.900 (0.303)</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="str">
+        <x:v>0.699 (0.329)</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="8" t="str">
-        <x:v>H1C0S1</x:v>
+        <x:v>H0C1S1</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>0.822 (0.218)</x:v>
+        <x:v>0.777 (0.270)</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>0.710 (0.272)</x:v>
+        <x:v>0.600 (0.321)</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>0.743 (0.281)</x:v>
+        <x:v>0.752 (0.301)</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>0.900 (0.303)</x:v>
+        <x:v>0.850 (0.360)</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>0.807 (0.200)</x:v>
+        <x:v>0.719 (0.218)</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="8" t="str">
-        <x:v>H1C1S0</x:v>
+        <x:v>H1C0S1</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>0.860 (0.181)</x:v>
+        <x:v>0.822 (0.218)</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>0.705 (0.248)</x:v>
+        <x:v>0.710 (0.272)</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>0.736 (0.271)</x:v>
+        <x:v>0.743 (0.281)</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>0.900 (0.303)</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>0.503 (0.229)</x:v>
+        <x:v>0.807 (0.200)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -3683,13 +3712,13 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>조건</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>평균(초)</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>SD(초)</x:v>
       </x:c>
     </x:row>
@@ -3810,25 +3839,25 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>지표</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>효과</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>df</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>p</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>보정 p</x:v>
       </x:c>
-      <x:c r="G3" s="6" t="str">
+      <x:c r="G3" s="10" t="str">
         <x:v>부분 η²</x:v>
       </x:c>
     </x:row>
@@ -3839,7 +3868,7 @@
       <x:c r="B4" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C4" s="8" t="str">
+      <x:c r="C4" s="9" t="str">
         <x:v>1, 57</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
@@ -3862,7 +3891,7 @@
       <x:c r="B5" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C5" s="8" t="str">
+      <x:c r="C5" s="9" t="str">
         <x:v>1, 57</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
@@ -3885,7 +3914,7 @@
       <x:c r="B6" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C6" s="8" t="str">
+      <x:c r="C6" s="9" t="str">
         <x:v>1, 57</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
@@ -3908,7 +3937,7 @@
       <x:c r="B7" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C7" s="8" t="str">
+      <x:c r="C7" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
@@ -3931,7 +3960,7 @@
       <x:c r="B8" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C8" s="8" t="str">
+      <x:c r="C8" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
@@ -3954,7 +3983,7 @@
       <x:c r="B9" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C9" s="8" t="str">
+      <x:c r="C9" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
@@ -3977,7 +4006,7 @@
       <x:c r="B10" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C10" s="8" t="str">
+      <x:c r="C10" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
@@ -4000,7 +4029,7 @@
       <x:c r="B11" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C11" s="8" t="str">
+      <x:c r="C11" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
@@ -4023,7 +4052,7 @@
       <x:c r="B12" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C12" s="8" t="str">
+      <x:c r="C12" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
@@ -4046,7 +4075,7 @@
       <x:c r="B13" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C13" s="8" t="str">
+      <x:c r="C13" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
@@ -4069,7 +4098,7 @@
       <x:c r="B14" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C14" s="8" t="str">
+      <x:c r="C14" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
@@ -4092,7 +4121,7 @@
       <x:c r="B15" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C15" s="8" t="str">
+      <x:c r="C15" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
@@ -4137,25 +4166,25 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>지표</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>효과</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>df</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>p</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>보정 p</x:v>
       </x:c>
-      <x:c r="G3" s="6" t="str">
+      <x:c r="G3" s="10" t="str">
         <x:v>부분 η²</x:v>
       </x:c>
     </x:row>
@@ -4166,7 +4195,7 @@
       <x:c r="B4" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C4" s="8" t="str">
+      <x:c r="C4" s="9" t="str">
         <x:v>1, 56</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
@@ -4189,7 +4218,7 @@
       <x:c r="B5" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C5" s="8" t="str">
+      <x:c r="C5" s="9" t="str">
         <x:v>1, 56</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
@@ -4212,7 +4241,7 @@
       <x:c r="B6" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C6" s="8" t="str">
+      <x:c r="C6" s="9" t="str">
         <x:v>1, 56</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
@@ -4235,7 +4264,7 @@
       <x:c r="B7" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C7" s="8" t="str">
+      <x:c r="C7" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
@@ -4258,7 +4287,7 @@
       <x:c r="B8" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C8" s="8" t="str">
+      <x:c r="C8" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
@@ -4281,7 +4310,7 @@
       <x:c r="B9" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C9" s="8" t="str">
+      <x:c r="C9" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
@@ -4304,7 +4333,7 @@
       <x:c r="B10" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C10" s="8" t="str">
+      <x:c r="C10" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
@@ -4327,7 +4356,7 @@
       <x:c r="B11" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C11" s="8" t="str">
+      <x:c r="C11" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
@@ -4350,7 +4379,7 @@
       <x:c r="B12" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C12" s="8" t="str">
+      <x:c r="C12" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
@@ -4373,7 +4402,7 @@
       <x:c r="B13" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="C13" s="8" t="str">
+      <x:c r="C13" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
@@ -4396,7 +4425,7 @@
       <x:c r="B14" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C14" s="8" t="str">
+      <x:c r="C14" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
@@ -4419,7 +4448,7 @@
       <x:c r="B15" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="C15" s="8" t="str">
+      <x:c r="C15" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
@@ -4463,22 +4492,22 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>효과</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>df</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>p</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>보정 p</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>부분 η²</x:v>
       </x:c>
     </x:row>
@@ -4486,7 +4515,7 @@
       <x:c r="A4" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B4" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
@@ -4506,7 +4535,7 @@
       <x:c r="A5" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="B5" s="8" t="str">
+      <x:c r="B5" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
@@ -4526,7 +4555,7 @@
       <x:c r="A6" s="8" t="str">
         <x:v>S</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="str">
+      <x:c r="B6" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
@@ -4546,7 +4575,7 @@
       <x:c r="A7" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="B7" s="8" t="str">
+      <x:c r="B7" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
@@ -4566,7 +4595,7 @@
       <x:c r="A8" s="8" t="str">
         <x:v>H×S</x:v>
       </x:c>
-      <x:c r="B8" s="8" t="str">
+      <x:c r="B8" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
@@ -4586,7 +4615,7 @@
       <x:c r="A9" s="8" t="str">
         <x:v>C×S</x:v>
       </x:c>
-      <x:c r="B9" s="8" t="str">
+      <x:c r="B9" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
@@ -4606,7 +4635,7 @@
       <x:c r="A10" s="8" t="str">
         <x:v>H×C×S</x:v>
       </x:c>
-      <x:c r="B10" s="8" t="str">
+      <x:c r="B10" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
@@ -4650,22 +4679,22 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>효과</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>df</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="D3" s="6" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>p</x:v>
       </x:c>
-      <x:c r="E3" s="6" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>보정 p</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>부분 η²</x:v>
       </x:c>
     </x:row>
@@ -4673,7 +4702,7 @@
       <x:c r="A4" s="8" t="str">
         <x:v>H</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B4" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
@@ -4693,7 +4722,7 @@
       <x:c r="A5" s="8" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="B5" s="8" t="str">
+      <x:c r="B5" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
@@ -4713,7 +4742,7 @@
       <x:c r="A6" s="8" t="str">
         <x:v>S</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="str">
+      <x:c r="B6" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
@@ -4733,7 +4762,7 @@
       <x:c r="A7" s="8" t="str">
         <x:v>H×C</x:v>
       </x:c>
-      <x:c r="B7" s="8" t="str">
+      <x:c r="B7" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
@@ -4753,7 +4782,7 @@
       <x:c r="A8" s="8" t="str">
         <x:v>H×S</x:v>
       </x:c>
-      <x:c r="B8" s="8" t="str">
+      <x:c r="B8" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
@@ -4773,7 +4802,7 @@
       <x:c r="A9" s="8" t="str">
         <x:v>C×S</x:v>
       </x:c>
-      <x:c r="B9" s="8" t="str">
+      <x:c r="B9" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
@@ -4793,7 +4822,7 @@
       <x:c r="A10" s="8" t="str">
         <x:v>H×C×S</x:v>
       </x:c>
-      <x:c r="B10" s="8" t="str">
+      <x:c r="B10" s="9" t="str">
         <x:v>1, 59</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">

</xml_diff>

<commit_message>
Finalize publication-grounded thesis and poster resubmission
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" r:id="R44db39e2cad547ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Factorial_Design" sheetId="2" r:id="R181d246532ba402b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="3" r:id="Reaae07f6769f4aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Mean_SD" sheetId="4" r:id="R28cfd973e48b477f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Runtime_SD" sheetId="5" r:id="Ra8b2ed1e3b1d4ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_Quality_S0" sheetId="6" r:id="R589fdbbea77744df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_Quality_S1" sheetId="7" r:id="Redd57846acee496a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_Factorial" sheetId="8" r:id="R6e277814193d4085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_Factorial" sheetId="9" r:id="Red3aba4d826b4810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-7_Paired_Quality" sheetId="10" r:id="R00c0d7aff4034723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-8_Paired_Language" sheetId="11" r:id="R79fc39bfe19b4fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="12" r:id="R7928e6df557f4bdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="13" r:id="R44d57f462e7447b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="14" r:id="Raa0122dce4e84a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2-1_Related_Work" sheetId="1" r:id="R09ef7c04f5434456"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3-1_Factorial_Design" sheetId="2" r:id="Rfce8f3e7f2a54759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4-1_Environment" sheetId="3" r:id="R5a725da41feb41f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-1_Mean_SD" sheetId="4" r:id="R19586b9c17864030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-2_Runtime_SD" sheetId="5" r:id="R6b2e1457d9b54083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-3_Quality_S0" sheetId="6" r:id="Rde833adaae9c4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-4_Quality_S1" sheetId="7" r:id="Rde8be6666838433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-5_Factorial" sheetId="8" r:id="R39bcd6bb04064dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-6_Factorial" sheetId="9" r:id="R8e8593a2a6194ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-7_Paired_Quality" sheetId="10" r:id="Rb1275b4139f149b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5-8_Paired_Language" sheetId="11" r:id="Rf485fc4b3b0e475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Queries" sheetId="12" r:id="Ra42016e2dd7344f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_Paper" sheetId="13" r:id="R21b66117d24247cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appendix_QueryType" sheetId="14" r:id="Rb38a9bcacf34490d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -411,18 +411,18 @@
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>Self-RAG[15], CRAG[16]</x:v>
+        <x:v>Self-RAG[15], Adaptive-RAG[16]</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>검색 및 근거 품질의 점검</x:v>
+        <x:v>자기평가 및 질문 복잡도에 따른 검색 전략 선택</x:v>
       </x:c>
       <x:c r="C8" s="7" t="str">
-        <x:v>검색 지표와 답변 지표를 구분하는 평가</x:v>
+        <x:v>고정 백본에서 입력·디코딩 조합의 효과 비교</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="7" t="str">
-        <x:v>RAGAS[10], BEIR[20], MTEB[21]</x:v>
+        <x:v>RAGAS[10], BEIR[19], MTEB[20]</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
         <x:v>자동 평가와 검색·임베딩 평가</x:v>

</xml_diff>

<commit_message>
Shorten table titles so the table of tables fits one line (v56)
The Hancom Web editor wrapped "ANOVA" in the table 5-3 and 5-4 entries
even though the PDF fitted them. Shorten the six titles with the least
room (5-1, 5-3, 5-4, 5-6, A-1, B-4) in the manuscript, table builder,
JSON and XLSX; re-export via Hancom (47 pages, anchors unchanged) and
record the change in the review report.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -600,7 +600,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 A-1 60개 한국어 질의의 대상 문서·유형·원문 페이지 및 정답 근거</t>
+          <t>표 A-1 60개 질의의 대상 문서·유형·원문 페이지·정답 근거</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 B-4 SCD ON 한국어 번역 평가의 품질 지표 H×C 반복측정 ANOVA</t>
+          <t>표 B-4 SCD ON 번역 평가의 품질 지표 H×C 반복측정 ANOVA</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 5-1 8조건의 품질 지표, 한국어 문자 비율과 실행 시간의 평균(SD)</t>
+          <t>표 5-1 8개 조건의 품질 지표·한국어 비율·실행 시간 평균(SD)</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 5-3 한국어 문자 비율에 대한 HyDE·CAD·SCD(H×C×S) 반복측정 ANOVA</t>
+          <t>표 5-3 한국어 문자 비율의 H×C×S 반복측정 ANOVA</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 5-4 조건 실행 시간에 대한 HyDE·CAD·SCD(H×C×S) 반복측정 ANOVA</t>
+          <t>표 5-4 실행 시간의 H×C×S 반복측정 ANOVA</t>
         </is>
       </c>
     </row>
@@ -6595,7 +6595,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 5-6 보조 지표(HyDE·CAD 품질, SCD 한국어 비율)의 대응 t-검정</t>
+          <t>표 5-6 HyDE·CAD 보조 지표와 SCD 한국어 비율의 대응 t-검정</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply the residual review and final layout check (v67)
- Define Cube-RAG as the study and Paper-RAG as its fixed pipeline (1.1)
- Retitle table 2-1 and its column, rewrite the table 5-6 lead-in
- Figure 1-1: "검색·생성 품질(RAGAS)"; figure 4-1: drop the duplicate
  definition line and cite only the reranker model [M2]
- Make the figure-usage section a subsection with its own page start
- 5.2 context precision as a rank-weighted score; split the 5.5 runtime
  paragraph and fix the median label; add the reranker scope to 5.9
- Tighten overlapping verbs in 3.2, 5.1, 5.3, 5.4
- Fix stale table counts and numbers in README, CURRENT_AUDIT and the
  poster README; mark PROSE_REVIEW as a historical record
- Rebuild HWPX, Hancom Web PDF v67 (47 pages), page map and manifest

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -445,7 +445,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>표 2-1 선행연구의 접근과 본 연구의 비교 질문</t>
+          <t>표 2-1 선행연구의 핵심 접근과 본 연구와의 관계</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>본 연구의 비교 질문</t>
+          <t>본 연구와의 관계</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revise thesis and poster around individual question profiles
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -912,12 +912,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>기준 평균</t>
+          <t>적용 전 평균</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>적용 평균</t>
+          <t>적용 후 평균</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -934,7 +934,8 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>영어 근거 평가 · 기준 미적용 → 적용 HyDE</t>
+          <t>기법 미적용 상태에서 HyDE만 적용했을 때의 답변 관련성
+영어 근거로 평가하였다. 관련성 0점이 있는 질문 9개를 제외하였다.</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -959,7 +960,7 @@
           <t>0.776</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>0.821</t>
         </is>
@@ -983,27 +984,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.575</t>
+          <t>0.726</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>0.747</t>
+          <t>0.795</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>+0.172</t>
+          <t>+0.069</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>14/3/12</t>
+          <t>8/2/12</t>
         </is>
       </c>
     </row>
@@ -1015,27 +1016,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>0.781</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>0.760</t>
+          <t>0.820</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>0.844</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>-0.022</t>
+          <t>+0.024</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>4/2/14</t>
+          <t>4/1/13</t>
         </is>
       </c>
     </row>
@@ -1079,34 +1080,35 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>0.683</t>
+          <t>0.772</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>0.763</t>
+          <t>0.816</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+0.080</t>
+          <t>+0.044</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>22/7/31</t>
+          <t>16/5/30</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>한국어 번역 근거 평가 · 기준 SCD → 적용 HyDE+SCD</t>
+          <t>SCD에 HyDE를 추가했을 때의 답변 관련성
+한국어로 번역한 근거로 평가하였다. 관련성 0점이 있는 질문 13개를 제외하였다.</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
@@ -1123,27 +1125,27 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>0.705</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>0.791</t>
+          <t>0.806</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>0.780</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>+0.086</t>
+          <t>-0.025</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>1/2/5</t>
+          <t>0/2/5</t>
         </is>
       </c>
     </row>
@@ -1155,27 +1157,27 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>0.531</t>
+          <t>0.722</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>0.688</t>
+          <t>0.767</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>+0.157</t>
+          <t>+0.045</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>12/7/10</t>
+          <t>6/5/9</t>
         </is>
       </c>
     </row>
@@ -1187,27 +1189,27 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>0.738</t>
+          <t>0.752</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>0.726</t>
+          <t>0.807</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>-0.012</t>
+          <t>+0.055</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>7/3/10</t>
+          <t>7/1/10</t>
         </is>
       </c>
     </row>
@@ -1219,27 +1221,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>0.808</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>0.595</t>
+          <t>0.918</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>0.892</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>-0.213</t>
+          <t>-0.026</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>0/2/1</t>
+          <t>0/1/1</t>
         </is>
       </c>
     </row>
@@ -1251,27 +1253,27 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>47</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>0.637</t>
+          <t>0.754</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>0.710</t>
+          <t>0.789</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>+0.072</t>
+          <t>+0.035</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>20/14/26</t>
+          <t>13/9/25</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1330,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>기준 평균</t>
+          <t>적용 전 평균</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>적용 평균</t>
+          <t>적용 후 평균</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -1350,7 +1352,8 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>영어 근거 평가 · 기준 미적용 → 적용 CAD</t>
+          <t>기법 미적용 상태에서 CAD만 적용했을 때의 근거 충실도
+영어 근거로 평가하였다.</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -1522,7 +1525,8 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>한국어 번역 근거 평가 · 기준 SCD → 적용 CAD+SCD</t>
+          <t>SCD에 CAD를 추가했을 때의 근거 충실도
+한국어로 번역한 근거로 평가하였다.</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
@@ -1744,12 +1748,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>기준 평균</t>
+          <t>적용 전 평균</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>적용 평균</t>
+          <t>적용 후 평균</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -1766,7 +1770,8 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>영어 근거 평가 · 기준 HyDE → 적용 HyDE+CAD</t>
+          <t>HyDE에 CAD를 추가했을 때의 답변 관련성
+영어 근거로 평가하였다. 관련성 0점이 있는 질문 7개를 제외하였다.</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -1791,7 +1796,7 @@
           <t>0.821</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>0.832</t>
         </is>
@@ -1815,27 +1820,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0.747</t>
+          <t>0.763</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.728</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>-0.104</t>
+          <t>-0.035</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>3/13/13</t>
+          <t>2/10/13</t>
         </is>
       </c>
     </row>
@@ -1847,27 +1852,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>0.760</t>
+          <t>0.844</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>0.760</t>
+          <t>0.808</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>+0.000</t>
+          <t>-0.036</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2/7/11</t>
+          <t>1/7/10</t>
         </is>
       </c>
     </row>
@@ -1879,27 +1884,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>0.788</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>0.586</t>
+          <t>0.873</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>0.880</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>-0.201</t>
+          <t>+0.006</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>0/1/2</t>
+          <t>0/0/2</t>
         </is>
       </c>
     </row>
@@ -1911,34 +1916,35 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>53</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>0.763</t>
+          <t>0.803</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>0.705</t>
+          <t>0.776</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>-0.059</t>
+          <t>-0.027</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>7/22/31</t>
+          <t>5/18/30</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>영어 근거 평가 · 기준 CAD → 적용 HyDE+CAD</t>
+          <t>CAD에 HyDE를 추가했을 때의 답변 관련성
+영어 근거로 평가하였다. 관련성 0점이 있는 질문 11개를 제외하였다.</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
@@ -1963,7 +1969,7 @@
           <t>0.761</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>0.832</t>
         </is>
@@ -1987,27 +1993,27 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.719</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>-0.001</t>
+          <t>-0.004</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>8/10/11</t>
+          <t>5/7/11</t>
         </is>
       </c>
     </row>
@@ -2019,27 +2025,27 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>0.713</t>
+          <t>0.797</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>0.760</t>
+          <t>0.799</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>+0.047</t>
+          <t>+0.002</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>3/2/15</t>
+          <t>1/1/15</t>
         </is>
       </c>
     </row>
@@ -2051,27 +2057,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>0.503</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>0.586</t>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>0.936</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+0.084</t>
+          <t>+0.000</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>1/1/1</t>
+          <t>0/0/1</t>
         </is>
       </c>
     </row>
@@ -2083,34 +2089,35 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>0.675</t>
+          <t>0.757</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>0.705</t>
+          <t>0.767</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>+0.029</t>
+          <t>+0.010</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>15/13/32</t>
+          <t>9/8/32</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>한국어 번역 근거 평가 · 기준 HyDE+SCD → 적용 HyDE+CAD+SCD</t>
+          <t>HyDE와 SCD에 CAD를 추가했을 때의 답변 관련성
+한국어로 번역한 근거로 평가하였다. 관련성 0점이 있는 질문 10개를 제외하였다.</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
@@ -2135,7 +2142,7 @@
           <t>0.791</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>0.781</t>
         </is>
@@ -2159,27 +2166,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>0.688</t>
+          <t>0.770</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>0.633</t>
+          <t>0.737</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>-0.055</t>
+          <t>-0.032</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>5/11/13</t>
+          <t>3/8/12</t>
         </is>
       </c>
     </row>
@@ -2191,27 +2198,27 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>0.726</t>
+          <t>0.834</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>0.684</t>
+          <t>0.804</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>-0.042</t>
+          <t>-0.030</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>1/6/13</t>
+          <t>1/5/11</t>
         </is>
       </c>
     </row>
@@ -2223,27 +2230,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>0.595</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>0.582</t>
+          <t>0.892</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>0.873</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>-0.013</t>
+          <t>-0.019</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>0/0/3</t>
+          <t>0/0/2</t>
         </is>
       </c>
     </row>
@@ -2255,34 +2262,35 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>0.710</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.773</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>-0.043</t>
+          <t>-0.027</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>7/18/35</t>
+          <t>5/14/31</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>한국어 번역 근거 평가 · 기준 CAD+SCD → 적용 HyDE+CAD+SCD</t>
+          <t>CAD와 SCD에 HyDE를 추가했을 때의 답변 관련성
+한국어로 번역한 근거로 평가하였다. 관련성 0점이 있는 질문 17개를 제외하였다.</t>
         </is>
       </c>
       <c r="B22" s="3" t="n"/>
@@ -2299,27 +2307,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>0.689</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>0.781</t>
+          <t>0.787</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>0.787</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>+0.092</t>
+          <t>+0.000</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>3/1/4</t>
+          <t>2/1/4</t>
         </is>
       </c>
     </row>
@@ -2331,27 +2339,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>0.530</t>
+          <t>0.707</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>0.633</t>
+          <t>0.723</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>+0.104</t>
+          <t>+0.016</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>10/7/12</t>
+          <t>4/4/11</t>
         </is>
       </c>
     </row>
@@ -2363,27 +2371,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>0.709</t>
+          <t>0.786</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>0.684</t>
+          <t>0.804</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>-0.025</t>
+          <t>+0.018</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>7/6/7</t>
+          <t>6/3/7</t>
         </is>
       </c>
     </row>
@@ -2395,27 +2403,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>0.312</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>0.582</t>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>0.936</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>+0.270</t>
+          <t>+0.000</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>1/0/2</t>
+          <t>0/0/1</t>
         </is>
       </c>
     </row>
@@ -2427,27 +2435,27 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>43</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.755</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.768</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>+0.067</t>
+          <t>+0.014</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>21/14/25</t>
+          <t>12/8/23</t>
         </is>
       </c>
     </row>
@@ -2506,29 +2514,30 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>정밀도 기준</t>
+          <t>정밀도 적용 전</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>정밀도 적용</t>
+          <t>정밀도 적용 후</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>재현율 기준</t>
+          <t>재현율 적용 전</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>재현율 적용</t>
+          <t>재현율 적용 후</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>영어 근거 평가 · 기준 미적용 → 적용 HyDE</t>
+          <t>기법 미적용 상태에서 HyDE만 적용했을 때의 검색 지표
+영어 근거로 평가하였다.</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -2700,7 +2709,8 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>한국어 번역 근거 평가 · 기준 SCD → 적용 HyDE+SCD</t>
+          <t>SCD에 HyDE를 추가했을 때의 검색 지표
+한국어로 번역한 근거로 평가하였다.</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
@@ -2922,12 +2932,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>기준 평균</t>
+          <t>적용 전 평균</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>적용 평균</t>
+          <t>적용 후 평균</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -2944,7 +2954,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>기준 미적용 → 적용 SCD</t>
+          <t>기법 미적용 상태에서 SCD만 적용했을 때의 한국어 문자 비율</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -3116,7 +3126,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>기준 HyDE → 적용 HyDE+SCD</t>
+          <t>HyDE에 SCD를 추가했을 때의 한국어 문자 비율</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
@@ -3288,7 +3298,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>기준 CAD → 적용 CAD+SCD</t>
+          <t>CAD에 SCD를 추가했을 때의 한국어 문자 비율</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
@@ -3460,7 +3470,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>기준 HyDE+CAD → 적용 HyDE+CAD+SCD</t>
+          <t>HyDE와 CAD에 SCD를 추가했을 때의 한국어 문자 비율</t>
         </is>
       </c>
       <c r="B22" s="3" t="n"/>
@@ -3684,12 +3694,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>기준 시간</t>
+          <t>적용 전 시간</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>적용 시간</t>
+          <t>적용 후 시간</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -3706,7 +3716,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>기준 미적용 → 적용 CAD</t>
+          <t>기법 미적용 상태에서 CAD만 적용했을 때의 처리 시간</t>
         </is>
       </c>
       <c r="B4" s="3" t="n"/>
@@ -3878,7 +3888,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>기준 미적용 → 적용 HyDE</t>
+          <t>기법 미적용 상태에서 HyDE만 적용했을 때의 처리 시간</t>
         </is>
       </c>
       <c r="B10" s="3" t="n"/>
@@ -4050,7 +4060,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>기준 미적용 → 적용 SCD</t>
+          <t>기법 미적용 상태에서 SCD만 적용했을 때의 처리 시간</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>

</xml_diff>

<commit_message>
Report thesis results with three decimals (v26)
The professor asked for three decimals in the thesis (10-18 recording,
AC-41) and two only on the poster (10-20 recording). Tables 5-1 and
5-2, appendix B scores, figures 4-2 and 5-2, and every result number in
chapters 4 to 6 are recomputed from the raw data with three decimals.
Two comparisons that were equal at two decimals now read as similar,
and the 5.6 context-precision range is corrected. Chapter 6 is trimmed
to stay on one page; Hancom v26 keeps 49 pages and every TOC anchor.
The A and B posters stay at two decimals and rebuild pixel-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FINALDOCS/TABLES/TABLES_60Q.xlsx
+++ b/FINALDOCS/TABLES/TABLES_60Q.xlsx
@@ -1257,38 +1257,38 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>0.79
-(0.26)</t>
+          <t>0.791
+(0.260)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>0.68
-(0.28)</t>
+          <t>0.683
+(0.282)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>0.75
-(0.30)</t>
+          <t>0.749
+(0.302)</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>0.93
-(0.25)</t>
+          <t>0.933
+(0.252)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>0.49
-(0.26)</t>
+          <t>0.494
+(0.265)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>16.66
-(5.05)</t>
+          <t>16.656
+(5.051)</t>
         </is>
       </c>
     </row>
@@ -1300,38 +1300,38 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>0.83
-(0.19)</t>
+          <t>0.834
+(0.186)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0.76
-(0.21)</t>
+          <t>0.763
+(0.209)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>0.71
-(0.30)</t>
+          <t>0.714
+(0.296)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>0.93
-(0.25)</t>
+          <t>0.933
+(0.252)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>0.56
-(0.21)</t>
+          <t>0.556
+(0.213)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>23.53
-(4.39)</t>
+          <t>23.533
+(4.385)</t>
         </is>
       </c>
     </row>
@@ -1343,38 +1343,38 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>0.84
-(0.20)</t>
+          <t>0.839
+(0.201)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>0.68
-(0.26)</t>
+          <t>0.675
+(0.261)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>0.74
-(0.30)</t>
+          <t>0.740
+(0.302)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>0.92
-(0.28)</t>
+          <t>0.917
+(0.279)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>0.49
-(0.24)</t>
+          <t>0.488
+(0.245)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>64.18
-(24.56)</t>
+          <t>64.182
+(24.563)</t>
         </is>
       </c>
     </row>
@@ -1386,38 +1386,38 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>0.79
-(0.25)</t>
+          <t>0.787
+(0.254)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>0.64
-(0.30)</t>
+          <t>0.637
+(0.296)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>0.76
-(0.30)</t>
+          <t>0.763
+(0.300)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>0.90
-(0.30)</t>
+          <t>0.900
+(0.303)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>0.70
-(0.33)</t>
+          <t>0.699
+(0.329)</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>18.66
-(5.00)</t>
+          <t>18.658
+(5.001)</t>
         </is>
       </c>
     </row>
@@ -1429,38 +1429,38 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>0.86
-(0.18)</t>
+          <t>0.860
+(0.181)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>0.70
-(0.25)</t>
+          <t>0.705
+(0.248)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0.74
-(0.27)</t>
+          <t>0.736
+(0.271)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>0.90
-(0.30)</t>
+          <t>0.900
+(0.303)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>0.50
-(0.23)</t>
+          <t>0.503
+(0.229)</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>72.53
-(21.24)</t>
+          <t>72.527
+(21.245)</t>
         </is>
       </c>
     </row>
@@ -1472,38 +1472,38 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>0.82
-(0.22)</t>
+          <t>0.822
+(0.218)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>0.71
-(0.27)</t>
+          <t>0.710
+(0.272)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>0.74
-(0.28)</t>
+          <t>0.743
+(0.281)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>0.90
-(0.30)</t>
+          <t>0.900
+(0.303)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>0.81
-(0.20)</t>
+          <t>0.807
+(0.200)</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>24.81
-(5.14)</t>
+          <t>24.811
+(5.145)</t>
         </is>
       </c>
     </row>
@@ -1515,38 +1515,38 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>0.78
-(0.27)</t>
+          <t>0.777
+(0.270)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>0.60
-(0.32)</t>
+          <t>0.600
+(0.321)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>0.75
-(0.30)</t>
+          <t>0.752
+(0.301)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>0.85
-(0.36)</t>
+          <t>0.850
+(0.360)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>0.72
-(0.22)</t>
+          <t>0.719
+(0.218)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>56.03
-(26.46)</t>
+          <t>56.033
+(26.463)</t>
         </is>
       </c>
     </row>
@@ -1558,38 +1558,38 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>0.83
-(0.25)</t>
+          <t>0.831
+(0.253)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>0.67
-(0.29)</t>
+          <t>0.667
+(0.286)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>0.75
-(0.27)</t>
+          <t>0.754
+(0.267)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>0.92
-(0.28)</t>
+          <t>0.917
+(0.279)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>0.73
-(0.21)</t>
+          <t>0.731
+(0.209)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>65.77
-(20.09)</t>
+          <t>65.770
+(20.091)</t>
         </is>
       </c>
     </row>
@@ -1698,32 +1698,32 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.826</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.726</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.848</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.743</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.575</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>0.78</t>
+          <t>0.778</t>
         </is>
       </c>
     </row>
@@ -1735,32 +1735,32 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.842</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>0.78</t>
+          <t>0.782</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.903</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.740</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.745</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>0.815</t>
         </is>
       </c>
     </row>
@@ -1772,32 +1772,32 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.896</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.830</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.789</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.752</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>0.63</t>
+          <t>0.629</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>0.66</t>
+          <t>0.663</t>
         </is>
       </c>
     </row>
@@ -1809,32 +1809,32 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.848</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.710</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>0.821</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.723</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.524</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.713</t>
         </is>
       </c>
     </row>
@@ -1846,32 +1846,32 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.927</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.796</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.882</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.761</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>0.63</t>
+          <t>0.630</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.755</t>
         </is>
       </c>
     </row>
@@ -1883,32 +1883,32 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.844</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.829</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.790</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.719</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.685</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.736</t>
         </is>
       </c>
     </row>
@@ -1920,32 +1920,32 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>0.77</t>
+          <t>0.767</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.761</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.809</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.719</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>0.503</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.616</t>
         </is>
       </c>
     </row>
@@ -1957,32 +1957,32 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.927</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.828</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.666</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>0.69</t>
+          <t>0.694</t>
         </is>
       </c>
     </row>
@@ -2054,32 +2054,32 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>0.67</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>0.73</t>
+          <t>0.668</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>0.730</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.862</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.944</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.880</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
@@ -2091,32 +2091,32 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.622</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.722</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.802</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.889</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>0.96</t>
+          <t>0.960</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.941</t>
         </is>
       </c>
     </row>
@@ -2128,32 +2128,32 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.670</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.734</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>0.821</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.889</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.880</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
@@ -2165,32 +2165,32 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>0.69</t>
+          <t>0.687</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.898</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.889</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.840</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
@@ -2202,32 +2202,32 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>0.68</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>0.73</t>
+          <t>0.680</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>0.729</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.804</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.944</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.840</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.941</t>
         </is>
       </c>
     </row>
@@ -2239,32 +2239,32 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.713</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>0.69</t>
+          <t>0.689</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.854</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.889</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.840</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
@@ -2276,32 +2276,32 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.677</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.729</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>0.87</t>
+          <t>0.867</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.941</t>
         </is>
       </c>
     </row>
@@ -2313,32 +2313,32 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.683</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.764</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.813</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>0.78</t>
+          <t>0.778</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>0.96</t>
+          <t>0.960</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
@@ -2410,32 +2410,32 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>0.58</t>
+          <t>0.585</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.455</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.456</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>14.65</t>
+          <t>14.648</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>16.66</t>
+          <t>16.662</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>18.91</t>
+          <t>18.906</t>
         </is>
       </c>
     </row>
@@ -2447,32 +2447,32 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.552</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.568</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.543</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>20.90</t>
+          <t>20.896</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>24.34</t>
+          <t>24.336</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>25.29</t>
+          <t>25.294</t>
         </is>
       </c>
     </row>
@@ -2484,32 +2484,32 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>0.417</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>0.504</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>55.41</t>
+          <t>55.410</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>67.12</t>
+          <t>67.124</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>69.64</t>
+          <t>69.636</t>
         </is>
       </c>
     </row>
@@ -2521,32 +2521,32 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.814</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>0.610</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.709</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>16.92</t>
+          <t>16.924</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>18.57</t>
+          <t>18.572</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>20.74</t>
+          <t>20.737</t>
         </is>
       </c>
     </row>
@@ -2558,32 +2558,32 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.520</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.458</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.552</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>60.59</t>
+          <t>60.591</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>78.75</t>
+          <t>78.747</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>76.62</t>
+          <t>76.623</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.835</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.785</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.810</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>24.07</t>
+          <t>24.065</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>23.74</t>
+          <t>23.737</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>27.26</t>
+          <t>27.262</t>
         </is>
       </c>
     </row>
@@ -2632,32 +2632,32 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>0.77</t>
+          <t>0.768</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.654</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.764</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>50.43</t>
+          <t>50.435</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>52.44</t>
+          <t>52.436</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>67.73</t>
+          <t>67.728</t>
         </is>
       </c>
     </row>
@@ -2669,32 +2669,32 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.737</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>0.69</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.789</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>59.86</t>
+          <t>59.862</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>64.91</t>
+          <t>64.909</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>73.71</t>
+          <t>73.706</t>
         </is>
       </c>
     </row>

</xml_diff>